<commit_message>
Corrección datos laboratorio . fecha análisis post corrección
</commit_message>
<xml_diff>
--- a/Datos Experimentales/Data 24018.xlsx
+++ b/Datos Experimentales/Data 24018.xlsx
@@ -1,7 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cltor\Documents\SB_Calibration_2025\Datos Experimentales\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D6FA4EF-F374-4BF4-94FE-2DB1B210BA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Antecedentes_info" sheetId="1" r:id="rId1"/>
     <sheet name="Antecedentes" sheetId="2" r:id="rId2"/>
@@ -18,6 +28,7 @@
     <sheet name="Manual Densidades" sheetId="13" r:id="rId13"/>
     <sheet name="Winegrid densidad" sheetId="14" r:id="rId14"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -1029,11 +1040,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1062,14 +1070,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1394,10 +1411,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B116"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1405,7 +1423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1413,7 +1431,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1421,7 +1439,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1429,7 +1447,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -1437,7 +1455,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -1445,7 +1463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -1453,7 +1471,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1461,7 +1479,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -1469,7 +1487,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -1477,7 +1495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -1485,7 +1503,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1493,7 +1511,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1501,7 +1519,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -1509,7 +1527,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1517,7 +1535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1525,7 +1543,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1533,7 +1551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1541,7 +1559,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1549,7 +1567,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -1557,7 +1575,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>23</v>
       </c>
@@ -1565,7 +1583,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1573,7 +1591,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -1581,7 +1599,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -1589,7 +1607,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -1597,7 +1615,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -1605,7 +1623,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>29</v>
       </c>
@@ -1613,7 +1631,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -1621,7 +1639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>31</v>
       </c>
@@ -1629,7 +1647,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -1637,7 +1655,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1645,7 +1663,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -1653,7 +1671,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -1661,7 +1679,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -1669,7 +1687,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1677,7 +1695,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1685,7 +1703,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1693,7 +1711,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1701,7 +1719,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1709,7 +1727,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1717,7 +1735,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1725,7 +1743,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -1733,7 +1751,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -1741,7 +1759,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1749,7 +1767,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -1757,7 +1775,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -1765,7 +1783,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1773,7 +1791,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>54</v>
       </c>
@@ -1781,7 +1799,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>55</v>
       </c>
@@ -1789,7 +1807,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>56</v>
       </c>
@@ -1797,7 +1815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>57</v>
       </c>
@@ -1805,7 +1823,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>58</v>
       </c>
@@ -1813,7 +1831,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>59</v>
       </c>
@@ -1821,7 +1839,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>61</v>
       </c>
@@ -1829,7 +1847,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>62</v>
       </c>
@@ -1837,7 +1855,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>63</v>
       </c>
@@ -1845,7 +1863,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>64</v>
       </c>
@@ -1853,7 +1871,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>65</v>
       </c>
@@ -1861,7 +1879,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>67</v>
       </c>
@@ -1869,7 +1887,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>68</v>
       </c>
@@ -1877,7 +1895,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -1885,7 +1903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>70</v>
       </c>
@@ -1893,7 +1911,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>71</v>
       </c>
@@ -1901,7 +1919,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>72</v>
       </c>
@@ -1909,7 +1927,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>73</v>
       </c>
@@ -1917,7 +1935,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>74</v>
       </c>
@@ -1925,7 +1943,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>75</v>
       </c>
@@ -1933,7 +1951,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>77</v>
       </c>
@@ -1941,7 +1959,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>78</v>
       </c>
@@ -1949,7 +1967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>79</v>
       </c>
@@ -1957,7 +1975,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>80</v>
       </c>
@@ -1965,7 +1983,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>81</v>
       </c>
@@ -1973,7 +1991,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>82</v>
       </c>
@@ -1981,7 +1999,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>83</v>
       </c>
@@ -1989,7 +2007,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>84</v>
       </c>
@@ -1997,7 +2015,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>85</v>
       </c>
@@ -2005,7 +2023,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>86</v>
       </c>
@@ -2013,7 +2031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>87</v>
       </c>
@@ -2021,7 +2039,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>89</v>
       </c>
@@ -2029,7 +2047,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>90</v>
       </c>
@@ -2037,7 +2055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>91</v>
       </c>
@@ -2045,7 +2063,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>93</v>
       </c>
@@ -2053,7 +2071,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>94</v>
       </c>
@@ -2061,7 +2079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>95</v>
       </c>
@@ -2069,7 +2087,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>96</v>
       </c>
@@ -2077,7 +2095,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>97</v>
       </c>
@@ -2085,7 +2103,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>98</v>
       </c>
@@ -2093,7 +2111,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>99</v>
       </c>
@@ -2101,7 +2119,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>100</v>
       </c>
@@ -2109,7 +2127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>101</v>
       </c>
@@ -2117,7 +2135,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>102</v>
       </c>
@@ -2125,7 +2143,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>103</v>
       </c>
@@ -2133,7 +2151,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>104</v>
       </c>
@@ -2141,7 +2159,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>105</v>
       </c>
@@ -2149,7 +2167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>106</v>
       </c>
@@ -2157,7 +2175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>107</v>
       </c>
@@ -2165,7 +2183,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>109</v>
       </c>
@@ -2173,7 +2191,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>110</v>
       </c>
@@ -2181,7 +2199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>111</v>
       </c>
@@ -2189,7 +2207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2197,7 +2215,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>113</v>
       </c>
@@ -2205,7 +2223,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>114</v>
       </c>
@@ -2213,7 +2231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>115</v>
       </c>
@@ -2221,7 +2239,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>116</v>
       </c>
@@ -2229,7 +2247,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>117</v>
       </c>
@@ -2237,7 +2255,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>118</v>
       </c>
@@ -2245,7 +2263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>119</v>
       </c>
@@ -2253,7 +2271,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>120</v>
       </c>
@@ -2261,7 +2279,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>121</v>
       </c>
@@ -2269,7 +2287,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>122</v>
       </c>
@@ -2277,7 +2295,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>123</v>
       </c>
@@ -2285,7 +2303,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>125</v>
       </c>
@@ -2293,7 +2311,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>126</v>
       </c>
@@ -2301,7 +2319,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>127</v>
       </c>
@@ -2309,7 +2327,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>128</v>
       </c>
@@ -2317,7 +2335,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>129</v>
       </c>
@@ -2326,27 +2344,31 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B116"/>
+    <ignoredError sqref="A1:B116" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>279</v>
       </c>
@@ -2367,17 +2389,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError sqref="A1:F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>284</v>
       </c>
@@ -2388,7 +2412,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>287</v>
       </c>
@@ -2399,7 +2423,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>288</v>
       </c>
@@ -2410,7 +2434,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>289</v>
       </c>
@@ -2421,7 +2445,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>290</v>
       </c>
@@ -2432,7 +2456,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>291</v>
       </c>
@@ -2443,7 +2467,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>292</v>
       </c>
@@ -2454,7 +2478,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>293</v>
       </c>
@@ -2465,7 +2489,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>294</v>
       </c>
@@ -2476,7 +2500,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>295</v>
       </c>
@@ -2487,7 +2511,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>296</v>
       </c>
@@ -2498,7 +2522,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>297</v>
       </c>
@@ -2509,7 +2533,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>298</v>
       </c>
@@ -2520,7 +2544,7 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>299</v>
       </c>
@@ -2531,7 +2555,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>300</v>
       </c>
@@ -2542,7 +2566,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>301</v>
       </c>
@@ -2550,10 +2574,10 @@
         <v>3.7416666666666667</v>
       </c>
       <c r="C16">
-        <v>16.6</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>16.600000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>302</v>
       </c>
@@ -2564,271 +2588,271 @@
         <v>17.5</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>303</v>
       </c>
       <c r="B18">
-        <v>4.241666666666667</v>
+        <v>4.2416666666666671</v>
       </c>
       <c r="C18">
-        <v>17.4</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>17.399999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>304</v>
       </c>
       <c r="B19">
-        <v>4.491666666666667</v>
+        <v>4.4916666666666671</v>
       </c>
       <c r="C19">
         <v>16.8</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>305</v>
       </c>
       <c r="B20">
-        <v>4.741666666666667</v>
+        <v>4.7416666666666671</v>
       </c>
       <c r="C20">
         <v>16.7</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>306</v>
       </c>
       <c r="B21">
-        <v>4.991666666666667</v>
+        <v>4.9916666666666671</v>
       </c>
       <c r="C21">
         <v>17.5</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>307</v>
       </c>
       <c r="B22">
-        <v>5.241666666666667</v>
+        <v>5.2416666666666671</v>
       </c>
       <c r="C22">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="23">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>308</v>
       </c>
       <c r="B23">
-        <v>5.491666666666667</v>
+        <v>5.4916666666666671</v>
       </c>
       <c r="C23">
         <v>16.5</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>309</v>
       </c>
       <c r="B24">
-        <v>5.741666666666667</v>
+        <v>5.7416666666666671</v>
       </c>
       <c r="C24">
         <v>17</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>310</v>
       </c>
       <c r="B25">
-        <v>5.991666666666667</v>
+        <v>5.9916666666666671</v>
       </c>
       <c r="C25">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>311</v>
       </c>
       <c r="B26">
-        <v>6.241666666666667</v>
+        <v>6.2416666666666671</v>
       </c>
       <c r="C26">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>312</v>
       </c>
       <c r="B27">
-        <v>6.491666666666667</v>
+        <v>6.4916666666666671</v>
       </c>
       <c r="C27">
         <v>17</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>313</v>
       </c>
       <c r="B28">
-        <v>6.741666666666667</v>
+        <v>6.7416666666666671</v>
       </c>
       <c r="C28">
         <v>17</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>314</v>
       </c>
       <c r="B29">
-        <v>6.991666666666667</v>
+        <v>6.9916666666666671</v>
       </c>
       <c r="C29">
         <v>16.5</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>315</v>
       </c>
       <c r="B30">
-        <v>7.241666666666667</v>
+        <v>7.2416666666666671</v>
       </c>
       <c r="C30">
         <v>17.2</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>316</v>
       </c>
       <c r="B31">
-        <v>7.491666666666667</v>
+        <v>7.4916666666666671</v>
       </c>
       <c r="C31">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="32">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>317</v>
       </c>
       <c r="B32">
-        <v>7.741666666666667</v>
+        <v>7.7416666666666671</v>
       </c>
       <c r="C32">
-        <v>17.6</v>
-      </c>
-    </row>
-    <row r="33">
+        <v>17.600000000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>318</v>
       </c>
       <c r="B33">
-        <v>7.991666666666667</v>
+        <v>7.9916666666666671</v>
       </c>
       <c r="C33">
         <v>17.7</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>319</v>
       </c>
       <c r="B34">
-        <v>8.241666666666667</v>
+        <v>8.2416666666666671</v>
       </c>
       <c r="C34">
         <v>16.8</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>320</v>
       </c>
       <c r="B35">
-        <v>8.491666666666667</v>
+        <v>8.4916666666666671</v>
       </c>
       <c r="C35">
         <v>17.7</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>321</v>
       </c>
       <c r="B36">
-        <v>8.741666666666667</v>
+        <v>8.7416666666666671</v>
       </c>
       <c r="C36">
         <v>17.2</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>322</v>
       </c>
       <c r="B37">
-        <v>8.991666666666667</v>
+        <v>8.9916666666666671</v>
       </c>
       <c r="C37">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="38">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>323</v>
       </c>
       <c r="B38">
-        <v>9.241666666666667</v>
+        <v>9.2416666666666671</v>
       </c>
       <c r="C38">
         <v>17.3</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>324</v>
       </c>
       <c r="B39">
-        <v>9.491666666666667</v>
+        <v>9.4916666666666671</v>
       </c>
       <c r="C39">
-        <v>17.9</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>17.899999999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>325</v>
       </c>
       <c r="B40">
-        <v>9.741666666666667</v>
+        <v>9.7416666666666671</v>
       </c>
       <c r="C40">
         <v>17.2</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>326</v>
       </c>
       <c r="B41">
-        <v>9.991666666666667</v>
+        <v>9.9916666666666671</v>
       </c>
       <c r="C41">
-        <v>16.9</v>
-      </c>
-    </row>
-    <row r="42">
+        <v>16.899999999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>327</v>
       </c>
@@ -2836,10 +2860,10 @@
         <v>10.241666666666667</v>
       </c>
       <c r="C42">
-        <v>17.1</v>
-      </c>
-    </row>
-    <row r="43">
+        <v>17.100000000000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>328</v>
       </c>
@@ -2850,7 +2874,7 @@
         <v>16.8</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>329</v>
       </c>
@@ -2861,7 +2885,7 @@
         <v>17.8</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>330</v>
       </c>
@@ -2869,21 +2893,23 @@
         <v>10.991666666666667</v>
       </c>
       <c r="C45">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
+    <ignoredError sqref="A1:C45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:C45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>284</v>
       </c>
@@ -2894,7 +2920,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>287</v>
       </c>
@@ -2905,7 +2931,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>288</v>
       </c>
@@ -2916,7 +2942,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>289</v>
       </c>
@@ -2927,7 +2953,7 @@
         <v>1085</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>290</v>
       </c>
@@ -2938,7 +2964,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>291</v>
       </c>
@@ -2949,7 +2975,7 @@
         <v>1084</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>292</v>
       </c>
@@ -2960,7 +2986,7 @@
         <v>1077</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>293</v>
       </c>
@@ -2971,7 +2997,7 @@
         <v>1073</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>294</v>
       </c>
@@ -2982,7 +3008,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>295</v>
       </c>
@@ -2993,7 +3019,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>296</v>
       </c>
@@ -3004,7 +3030,7 @@
         <v>1052</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>297</v>
       </c>
@@ -3015,7 +3041,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>298</v>
       </c>
@@ -3026,7 +3052,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>299</v>
       </c>
@@ -3037,7 +3063,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>300</v>
       </c>
@@ -3048,7 +3074,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>301</v>
       </c>
@@ -3059,7 +3085,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>302</v>
       </c>
@@ -3070,271 +3096,271 @@
         <v>1027</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>303</v>
       </c>
       <c r="B18">
-        <v>4.241666666666667</v>
+        <v>4.2416666666666671</v>
       </c>
       <c r="C18">
         <v>1023</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>304</v>
       </c>
       <c r="B19">
-        <v>4.491666666666667</v>
+        <v>4.4916666666666671</v>
       </c>
       <c r="C19">
         <v>1020</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>305</v>
       </c>
       <c r="B20">
-        <v>4.741666666666667</v>
+        <v>4.7416666666666671</v>
       </c>
       <c r="C20">
         <v>1018</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>306</v>
       </c>
       <c r="B21">
-        <v>4.991666666666667</v>
+        <v>4.9916666666666671</v>
       </c>
       <c r="C21">
         <v>1015</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>307</v>
       </c>
       <c r="B22">
-        <v>5.241666666666667</v>
+        <v>5.2416666666666671</v>
       </c>
       <c r="C22">
         <v>1015</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>308</v>
       </c>
       <c r="B23">
-        <v>5.491666666666667</v>
+        <v>5.4916666666666671</v>
       </c>
       <c r="C23">
         <v>1012</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>309</v>
       </c>
       <c r="B24">
-        <v>5.741666666666667</v>
+        <v>5.7416666666666671</v>
       </c>
       <c r="C24">
         <v>1008</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>310</v>
       </c>
       <c r="B25">
-        <v>5.991666666666667</v>
+        <v>5.9916666666666671</v>
       </c>
       <c r="C25">
         <v>1006</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>311</v>
       </c>
       <c r="B26">
-        <v>6.241666666666667</v>
+        <v>6.2416666666666671</v>
       </c>
       <c r="C26">
         <v>1007</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>312</v>
       </c>
       <c r="B27">
-        <v>6.491666666666667</v>
+        <v>6.4916666666666671</v>
       </c>
       <c r="C27">
         <v>1004</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>313</v>
       </c>
       <c r="B28">
-        <v>6.741666666666667</v>
+        <v>6.7416666666666671</v>
       </c>
       <c r="C28">
         <v>1003</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>314</v>
       </c>
       <c r="B29">
-        <v>6.991666666666667</v>
+        <v>6.9916666666666671</v>
       </c>
       <c r="C29">
         <v>1003</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>315</v>
       </c>
       <c r="B30">
-        <v>7.241666666666667</v>
+        <v>7.2416666666666671</v>
       </c>
       <c r="C30">
         <v>1003</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>316</v>
       </c>
       <c r="B31">
-        <v>7.491666666666667</v>
+        <v>7.4916666666666671</v>
       </c>
       <c r="C31">
         <v>1000</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>317</v>
       </c>
       <c r="B32">
-        <v>7.741666666666667</v>
+        <v>7.7416666666666671</v>
       </c>
       <c r="C32">
         <v>1000</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>318</v>
       </c>
       <c r="B33">
-        <v>7.991666666666667</v>
+        <v>7.9916666666666671</v>
       </c>
       <c r="C33">
         <v>999</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>319</v>
       </c>
       <c r="B34">
-        <v>8.241666666666667</v>
+        <v>8.2416666666666671</v>
       </c>
       <c r="C34">
         <v>999</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>320</v>
       </c>
       <c r="B35">
-        <v>8.491666666666667</v>
+        <v>8.4916666666666671</v>
       </c>
       <c r="C35">
         <v>996</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>321</v>
       </c>
       <c r="B36">
-        <v>8.741666666666667</v>
+        <v>8.7416666666666671</v>
       </c>
       <c r="C36">
         <v>997</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>322</v>
       </c>
       <c r="B37">
-        <v>8.991666666666667</v>
+        <v>8.9916666666666671</v>
       </c>
       <c r="C37">
         <v>997</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>323</v>
       </c>
       <c r="B38">
-        <v>9.241666666666667</v>
+        <v>9.2416666666666671</v>
       </c>
       <c r="C38">
         <v>997</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>324</v>
       </c>
       <c r="B39">
-        <v>9.491666666666667</v>
+        <v>9.4916666666666671</v>
       </c>
       <c r="C39">
         <v>995</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>325</v>
       </c>
       <c r="B40">
-        <v>9.741666666666667</v>
+        <v>9.7416666666666671</v>
       </c>
       <c r="C40">
         <v>995</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>326</v>
       </c>
       <c r="B41">
-        <v>9.991666666666667</v>
+        <v>9.9916666666666671</v>
       </c>
       <c r="C41">
         <v>994</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>327</v>
       </c>
@@ -3345,7 +3371,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>328</v>
       </c>
@@ -3356,7 +3382,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>329</v>
       </c>
@@ -3367,7 +3393,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>330</v>
       </c>
@@ -3379,17 +3405,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C45"/>
+    <ignoredError sqref="A1:C45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>284</v>
       </c>
@@ -3413,17 +3441,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError sqref="A1:G1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:CY2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:103" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3734,7 +3764,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:103" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -3769,7 +3799,7 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>45373.63333333333</v>
+        <v>45373.633333333331</v>
       </c>
       <c r="M2" t="s">
         <v>134</v>
@@ -3778,7 +3808,7 @@
         <v>135</v>
       </c>
       <c r="O2">
-        <v>45379.63333333333</v>
+        <v>45379.633333333331</v>
       </c>
       <c r="P2" t="s">
         <v>136</v>
@@ -3859,7 +3889,7 @@
         <v>144</v>
       </c>
       <c r="AS2">
-        <v>17.4</v>
+        <v>17.399999999999999</v>
       </c>
       <c r="AT2">
         <v>11.6</v>
@@ -3955,7 +3985,7 @@
         <v>0</v>
       </c>
       <c r="BY2">
-        <v>0.014</v>
+        <v>1.4E-2</v>
       </c>
       <c r="BZ2">
         <v>0</v>
@@ -3997,7 +4027,7 @@
         <v>0</v>
       </c>
       <c r="CM2">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="CN2">
         <v>0</v>
@@ -4025,17 +4055,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:CY2"/>
+    <ignoredError sqref="A1:CY2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>160</v>
       </c>
@@ -4088,7 +4120,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -4117,7 +4149,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9838</v>
       </c>
@@ -4152,7 +4184,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9838</v>
       </c>
@@ -4181,7 +4213,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9838</v>
       </c>
@@ -4195,7 +4227,7 @@
         <v>185</v>
       </c>
       <c r="E5">
-        <v>0.014</v>
+        <v>1.4E-2</v>
       </c>
       <c r="F5" t="s">
         <v>181</v>
@@ -4231,7 +4263,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9838</v>
       </c>
@@ -4245,7 +4277,7 @@
         <v>185</v>
       </c>
       <c r="E6">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="F6" t="s">
         <v>181</v>
@@ -4281,7 +4313,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9838</v>
       </c>
@@ -4316,7 +4348,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9838</v>
       </c>
@@ -4363,7 +4395,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9838</v>
       </c>
@@ -4392,7 +4424,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9838</v>
       </c>
@@ -4427,7 +4459,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9838</v>
       </c>
@@ -4462,7 +4494,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9838</v>
       </c>
@@ -4498,17 +4530,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q12"/>
+    <ignoredError sqref="A1:Q12" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:J4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>160</v>
       </c>
@@ -4540,7 +4574,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -4572,7 +4606,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9838</v>
       </c>
@@ -4604,7 +4638,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9838</v>
       </c>
@@ -4637,27 +4671,31 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError sqref="A1:J4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>160</v>
       </c>
@@ -4689,7 +4727,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -4722,17 +4760,19 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError sqref="A1:J2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>160</v>
       </c>
@@ -4749,7 +4789,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -4761,27 +4801,31 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError sqref="A1:E2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError sqref="A1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:P36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>160</v>
       </c>
@@ -4831,7 +4875,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>9838</v>
       </c>
@@ -4844,8 +4888,8 @@
       <c r="D2">
         <v>6811</v>
       </c>
-      <c r="E2">
-        <v>45373.76887731481</v>
+      <c r="E2" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F2" t="s">
         <v>133</v>
@@ -4875,13 +4919,13 @@
         <v>243</v>
       </c>
       <c r="O2">
-        <v>7.5735</v>
+        <v>7.5735000000000001</v>
       </c>
       <c r="P2" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>9838</v>
       </c>
@@ -4894,8 +4938,8 @@
       <c r="D3">
         <v>6811</v>
       </c>
-      <c r="E3">
-        <v>45373.76887731481</v>
+      <c r="E3" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F3" t="s">
         <v>133</v>
@@ -4925,13 +4969,13 @@
         <v>243</v>
       </c>
       <c r="O3">
-        <v>3.435</v>
+        <v>3.4350000000000001</v>
       </c>
       <c r="P3" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>9838</v>
       </c>
@@ -4944,8 +4988,8 @@
       <c r="D4">
         <v>6811</v>
       </c>
-      <c r="E4">
-        <v>45373.76887731481</v>
+      <c r="E4" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F4" t="s">
         <v>133</v>
@@ -4981,7 +5025,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>9838</v>
       </c>
@@ -4994,8 +5038,8 @@
       <c r="D5">
         <v>6811</v>
       </c>
-      <c r="E5">
-        <v>45373.76887731481</v>
+      <c r="E5" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F5" t="s">
         <v>133</v>
@@ -5031,7 +5075,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>9838</v>
       </c>
@@ -5044,8 +5088,8 @@
       <c r="D6">
         <v>6811</v>
       </c>
-      <c r="E6">
-        <v>45373.76887731481</v>
+      <c r="E6" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F6" t="s">
         <v>133</v>
@@ -5081,7 +5125,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>9838</v>
       </c>
@@ -5094,8 +5138,8 @@
       <c r="D7">
         <v>6811</v>
       </c>
-      <c r="E7">
-        <v>45373.76887731481</v>
+      <c r="E7" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F7" t="s">
         <v>133</v>
@@ -5131,7 +5175,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>9838</v>
       </c>
@@ -5144,8 +5188,8 @@
       <c r="D8">
         <v>6811</v>
       </c>
-      <c r="E8">
-        <v>45373.76887731481</v>
+      <c r="E8" s="1">
+        <v>45373.768877314811</v>
       </c>
       <c r="F8" t="s">
         <v>133</v>
@@ -5181,7 +5225,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>9838</v>
       </c>
@@ -5194,8 +5238,8 @@
       <c r="D9">
         <v>6878</v>
       </c>
-      <c r="E9">
-        <v>45376.65599537037</v>
+      <c r="E9" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F9" t="s">
         <v>133</v>
@@ -5225,13 +5269,13 @@
         <v>243</v>
       </c>
       <c r="O9">
-        <v>8.0019</v>
+        <v>8.0018999999999991</v>
       </c>
       <c r="P9" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9838</v>
       </c>
@@ -5244,8 +5288,8 @@
       <c r="D10">
         <v>6878</v>
       </c>
-      <c r="E10">
-        <v>45376.65599537037</v>
+      <c r="E10" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F10" t="s">
         <v>133</v>
@@ -5281,7 +5325,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9838</v>
       </c>
@@ -5294,8 +5338,8 @@
       <c r="D11">
         <v>6878</v>
       </c>
-      <c r="E11">
-        <v>45376.65599537037</v>
+      <c r="E11" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F11" t="s">
         <v>133</v>
@@ -5331,7 +5375,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>9838</v>
       </c>
@@ -5344,8 +5388,8 @@
       <c r="D12">
         <v>6878</v>
       </c>
-      <c r="E12">
-        <v>45376.65599537037</v>
+      <c r="E12" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F12" t="s">
         <v>133</v>
@@ -5381,7 +5425,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>9838</v>
       </c>
@@ -5394,8 +5438,8 @@
       <c r="D13">
         <v>6878</v>
       </c>
-      <c r="E13">
-        <v>45376.65599537037</v>
+      <c r="E13" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F13" t="s">
         <v>133</v>
@@ -5431,7 +5475,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>9838</v>
       </c>
@@ -5444,8 +5488,8 @@
       <c r="D14">
         <v>6878</v>
       </c>
-      <c r="E14">
-        <v>45376.65599537037</v>
+      <c r="E14" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F14" t="s">
         <v>133</v>
@@ -5481,7 +5525,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>9838</v>
       </c>
@@ -5494,8 +5538,8 @@
       <c r="D15">
         <v>6878</v>
       </c>
-      <c r="E15">
-        <v>45376.65599537037</v>
+      <c r="E15" s="1">
+        <v>45373.655995370369</v>
       </c>
       <c r="F15" t="s">
         <v>133</v>
@@ -5531,7 +5575,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>9838</v>
       </c>
@@ -5544,8 +5588,8 @@
       <c r="D16">
         <v>7095</v>
       </c>
-      <c r="E16">
-        <v>45383.62201388889</v>
+      <c r="E16" s="1">
+        <v>45383.622013888889</v>
       </c>
       <c r="F16" t="s">
         <v>133</v>
@@ -5581,7 +5625,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>9838</v>
       </c>
@@ -5594,7 +5638,7 @@
       <c r="D17">
         <v>7096</v>
       </c>
-      <c r="E17">
+      <c r="E17" s="1">
         <v>45383.622037037036</v>
       </c>
       <c r="F17" t="s">
@@ -5631,7 +5675,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>9838</v>
       </c>
@@ -5644,8 +5688,8 @@
       <c r="D18">
         <v>7161</v>
       </c>
-      <c r="E18">
-        <v>45384.8509375</v>
+      <c r="E18" s="1">
+        <v>45384.850937499999</v>
       </c>
       <c r="F18" t="s">
         <v>133</v>
@@ -5681,7 +5725,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>9838</v>
       </c>
@@ -5694,8 +5738,8 @@
       <c r="D19">
         <v>7243</v>
       </c>
-      <c r="E19">
-        <v>45386.86607638889</v>
+      <c r="E19" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F19" t="s">
         <v>133</v>
@@ -5731,7 +5775,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>9838</v>
       </c>
@@ -5744,8 +5788,8 @@
       <c r="D20">
         <v>7243</v>
       </c>
-      <c r="E20">
-        <v>45386.86607638889</v>
+      <c r="E20" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F20" t="s">
         <v>133</v>
@@ -5781,7 +5825,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>9838</v>
       </c>
@@ -5794,8 +5838,8 @@
       <c r="D21">
         <v>7243</v>
       </c>
-      <c r="E21">
-        <v>45386.86607638889</v>
+      <c r="E21" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F21" t="s">
         <v>133</v>
@@ -5831,7 +5875,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>9838</v>
       </c>
@@ -5844,8 +5888,8 @@
       <c r="D22">
         <v>7243</v>
       </c>
-      <c r="E22">
-        <v>45386.86607638889</v>
+      <c r="E22" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F22" t="s">
         <v>133</v>
@@ -5881,7 +5925,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>9838</v>
       </c>
@@ -5894,8 +5938,8 @@
       <c r="D23">
         <v>7243</v>
       </c>
-      <c r="E23">
-        <v>45386.86607638889</v>
+      <c r="E23" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F23" t="s">
         <v>133</v>
@@ -5925,13 +5969,13 @@
         <v>243</v>
       </c>
       <c r="O23">
-        <v>0.137</v>
+        <v>0.13700000000000001</v>
       </c>
       <c r="P23" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>9838</v>
       </c>
@@ -5944,8 +5988,8 @@
       <c r="D24">
         <v>7243</v>
       </c>
-      <c r="E24">
-        <v>45386.86607638889</v>
+      <c r="E24" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F24" t="s">
         <v>133</v>
@@ -5981,7 +6025,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>9838</v>
       </c>
@@ -5994,8 +6038,8 @@
       <c r="D25">
         <v>7243</v>
       </c>
-      <c r="E25">
-        <v>45386.86607638889</v>
+      <c r="E25" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F25" t="s">
         <v>133</v>
@@ -6031,7 +6075,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>9838</v>
       </c>
@@ -6044,8 +6088,8 @@
       <c r="D26">
         <v>7243</v>
       </c>
-      <c r="E26">
-        <v>45386.86607638889</v>
+      <c r="E26" s="1">
+        <v>45386.866076388891</v>
       </c>
       <c r="F26" t="s">
         <v>133</v>
@@ -6081,7 +6125,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>9838</v>
       </c>
@@ -6094,8 +6138,8 @@
       <c r="D27">
         <v>7245</v>
       </c>
-      <c r="E27">
-        <v>45386.86703703704</v>
+      <c r="E27" s="1">
+        <v>45386.867037037038</v>
       </c>
       <c r="F27" t="s">
         <v>133</v>
@@ -6131,7 +6175,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>9838</v>
       </c>
@@ -6144,7 +6188,7 @@
       <c r="D28">
         <v>7266</v>
       </c>
-      <c r="E28">
+      <c r="E28" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F28" t="s">
@@ -6181,7 +6225,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>9838</v>
       </c>
@@ -6194,7 +6238,7 @@
       <c r="D29">
         <v>7266</v>
       </c>
-      <c r="E29">
+      <c r="E29" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F29" t="s">
@@ -6231,7 +6275,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>9838</v>
       </c>
@@ -6244,7 +6288,7 @@
       <c r="D30">
         <v>7266</v>
       </c>
-      <c r="E30">
+      <c r="E30" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F30" t="s">
@@ -6281,7 +6325,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>9838</v>
       </c>
@@ -6294,7 +6338,7 @@
       <c r="D31">
         <v>7266</v>
       </c>
-      <c r="E31">
+      <c r="E31" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F31" t="s">
@@ -6331,7 +6375,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>9838</v>
       </c>
@@ -6344,7 +6388,7 @@
       <c r="D32">
         <v>7266</v>
       </c>
-      <c r="E32">
+      <c r="E32" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F32" t="s">
@@ -6381,7 +6425,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>9838</v>
       </c>
@@ -6394,7 +6438,7 @@
       <c r="D33">
         <v>7266</v>
       </c>
-      <c r="E33">
+      <c r="E33" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F33" t="s">
@@ -6425,13 +6469,13 @@
         <v>243</v>
       </c>
       <c r="O33">
-        <v>0.165</v>
+        <v>0.16500000000000001</v>
       </c>
       <c r="P33" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>9838</v>
       </c>
@@ -6444,7 +6488,7 @@
       <c r="D34">
         <v>7266</v>
       </c>
-      <c r="E34">
+      <c r="E34" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F34" t="s">
@@ -6481,7 +6525,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>9838</v>
       </c>
@@ -6494,7 +6538,7 @@
       <c r="D35">
         <v>7266</v>
       </c>
-      <c r="E35">
+      <c r="E35" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F35" t="s">
@@ -6531,7 +6575,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>9838</v>
       </c>
@@ -6544,7 +6588,7 @@
       <c r="D36">
         <v>7266</v>
       </c>
-      <c r="E36">
+      <c r="E36" s="1">
         <v>45387.60728009259</v>
       </c>
       <c r="F36" t="s">
@@ -6582,8 +6626,9 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P36"/>
+    <ignoredError sqref="A1:P8 A16:P36 A9:D9 F9:P9 A10:D15 F10:P15" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>